<commit_message>
Updated Ads consent to official Google Flow
</commit_message>
<xml_diff>
--- a/výpočty_rozložení.xlsx
+++ b/výpočty_rozložení.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uzivatel\Desktop\Projekty\Tetros\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uzivatel\Desktop\Projekty\SharpStack\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3CB594E-B59D-432C-ADB6-8F279815B8A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E542F6-EF0A-4CE7-BF1F-44B82778901C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6255" yWindow="4830" windowWidth="23010" windowHeight="12210" xr2:uid="{48DBA291-C9C2-471D-9B40-A2E682837783}"/>
+    <workbookView xWindow="12" yWindow="12" windowWidth="23016" windowHeight="12216" xr2:uid="{48DBA291-C9C2-471D-9B40-A2E682837783}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>Co</t>
   </si>
@@ -100,6 +99,9 @@
   </si>
   <si>
     <t>Score_Text</t>
+  </si>
+  <si>
+    <t>nextBrick</t>
   </si>
 </sst>
 </file>
@@ -476,6 +478,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="12.5703125" customWidth="1"/>
     <col min="9" max="9" width="12.28515625" customWidth="1"/>
     <col min="10" max="10" width="13.42578125" customWidth="1"/>
@@ -565,7 +569,7 @@
       </c>
       <c r="C4">
         <f>$E$3+$C$3+I4</f>
-        <v>2048</v>
+        <v>1990</v>
       </c>
       <c r="D4">
         <v>200</v>
@@ -579,13 +583,13 @@
       </c>
       <c r="G4">
         <f t="shared" ref="G4:G13" si="1">C4+E4</f>
-        <v>2248</v>
+        <v>2190</v>
       </c>
       <c r="H4">
         <v>100</v>
       </c>
       <c r="I4">
-        <v>358</v>
+        <v>300</v>
       </c>
       <c r="J4" t="s">
         <v>17</v>
@@ -601,7 +605,7 @@
       </c>
       <c r="C5">
         <f t="shared" ref="C5:C7" si="2">$E$3+$C$3+I5</f>
-        <v>2048</v>
+        <v>1990</v>
       </c>
       <c r="D5">
         <v>200</v>
@@ -615,13 +619,13 @@
       </c>
       <c r="G5">
         <f t="shared" si="1"/>
-        <v>2248</v>
+        <v>2190</v>
       </c>
       <c r="H5">
         <v>-100</v>
       </c>
       <c r="I5">
-        <v>358</v>
+        <v>300</v>
       </c>
       <c r="J5" t="s">
         <v>18</v>
@@ -637,7 +641,7 @@
       </c>
       <c r="C6">
         <f t="shared" si="2"/>
-        <v>1769</v>
+        <v>1740</v>
       </c>
       <c r="D6">
         <v>200</v>
@@ -651,13 +655,13 @@
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>1969</v>
+        <v>1940</v>
       </c>
       <c r="H6">
         <v>100</v>
       </c>
       <c r="I6">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="J6" t="s">
         <v>17</v>
@@ -673,7 +677,7 @@
       </c>
       <c r="C7">
         <f t="shared" si="2"/>
-        <v>1769</v>
+        <v>1740</v>
       </c>
       <c r="D7">
         <v>200</v>
@@ -687,13 +691,13 @@
       </c>
       <c r="G7">
         <f t="shared" si="1"/>
-        <v>1969</v>
+        <v>1940</v>
       </c>
       <c r="H7">
         <v>-100</v>
       </c>
       <c r="I7">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="J7" t="s">
         <v>18</v>
@@ -707,7 +711,7 @@
         <v>540</v>
       </c>
       <c r="C8">
-        <v>1800</v>
+        <v>1770</v>
       </c>
       <c r="D8" t="s">
         <v>6</v>
@@ -725,13 +729,22 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9">
+        <v>515</v>
+      </c>
+      <c r="C9">
+        <v>2000</v>
+      </c>
       <c r="F9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>515</v>
       </c>
       <c r="G9">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>